<commit_message>
Update notebook and model results
</commit_message>
<xml_diff>
--- a/potato_yield_model_results.xlsx
+++ b/potato_yield_model_results.xlsx
@@ -482,7 +482,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Stepwise Linear Regression</t>
+          <t>Multiple Linear Regression</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -573,7 +573,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Stepwise Linear Regression</t>
+          <t>Multiple Linear Regression</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">

</xml_diff>